<commit_message>
feat(content-runtime): G01-P7-M10 preserve exact per-hit payloads
</commit_message>
<xml_diff>
--- a/config/data/HitPlanHit.xlsx
+++ b/config/data/HitPlanHit.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -24,16 +24,68 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF1F2937"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F3A4A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9EEF5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3D6E8F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDE5EF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8FB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7DB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -41,12 +93,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -414,237 +499,340 @@
   </sheetPr>
   <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12.7109375" customWidth="1" min="1" max="1"/>
+    <col width="15.7109375" customWidth="1" style="5" min="2" max="2"/>
+    <col width="12.7109375" customWidth="1" style="5" min="3" max="3"/>
+    <col width="20.7109375" customWidth="1" style="5" min="4" max="5"/>
+    <col width="23.7109375" customWidth="1" style="5" min="6" max="6"/>
+    <col width="16.7109375" customWidth="1" style="5" min="7" max="7"/>
+    <col width="29.7109375" customWidth="1" style="5" min="8" max="8"/>
+    <col width="30.7109375" customWidth="1" style="5" min="9" max="9"/>
+    <col width="24.7109375" customWidth="1" style="5" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>@table</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>HitPlanHit</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>@mode</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>list</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>@key</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>@scope</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>@schema</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>df0d9f01c3e44551</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>ba104ad9faac7ac3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>#name</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>hit_plan_id</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>sequence</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>target_group</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>damage_ratio_decimal</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>toughness_ratio_decimal</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>crit_policy</t>
         </is>
       </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>damage_parameter_key_override</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>damage_operation_ratio_decimal</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>toughness_amount_decimal</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>#field</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>hit_plan_id</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>sequence</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>target_group</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>damage_ratio_decimal</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>toughness_ratio_decimal</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>crit_policy</t>
         </is>
       </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>damage_parameter_key_override</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>damage_operation_ratio_decimal</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>toughness_amount_decimal</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>#type</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>ref&lt;HitPlan.id&gt;</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>i32</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>enum&lt;HitTargetGroup&gt;</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>string</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>enum&lt;CritPolicy&gt;</t>
         </is>
       </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>optional&lt;string&gt;</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>optional&lt;string&gt;</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>optional&lt;string&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>#scope</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>#input</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>range=1..100</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>length=1..32</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>length=1..32</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>length=1..120</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>length=1..32</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>length=1..32</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>#desc</t>
         </is>
       </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" t="n">
-        <v>12001</v>
-      </c>
-      <c r="C8" t="n">
-        <v>1</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>12001</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -668,11 +856,15 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" t="n">
-        <v>12003</v>
-      </c>
-      <c r="C9" t="n">
-        <v>1</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>12003</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -696,11 +888,15 @@
       </c>
     </row>
     <row r="10">
-      <c r="B10" t="n">
-        <v>12004</v>
-      </c>
-      <c r="C10" t="n">
-        <v>1</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>12004</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -724,11 +920,15 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" t="n">
-        <v>12006</v>
-      </c>
-      <c r="C11" t="n">
-        <v>1</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>12006</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -752,11 +952,15 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" t="n">
-        <v>12007</v>
-      </c>
-      <c r="C12" t="n">
-        <v>1</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>12007</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -780,11 +984,15 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" t="n">
-        <v>12008</v>
-      </c>
-      <c r="C13" t="n">
-        <v>1</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>12008</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -808,11 +1016,15 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" t="n">
-        <v>12009</v>
-      </c>
-      <c r="C14" t="n">
-        <v>1</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>12009</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -836,11 +1048,15 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" t="n">
-        <v>12012</v>
-      </c>
-      <c r="C15" t="n">
-        <v>1</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>12012</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -864,11 +1080,15 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" t="n">
-        <v>12013</v>
-      </c>
-      <c r="C16" t="n">
-        <v>1</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>12013</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -892,11 +1112,15 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" t="n">
-        <v>12014</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1</v>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>12014</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -920,11 +1144,15 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" t="n">
-        <v>12017</v>
-      </c>
-      <c r="C18" t="n">
-        <v>1</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>12017</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -948,11 +1176,15 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" t="n">
-        <v>12018</v>
-      </c>
-      <c r="C19" t="n">
-        <v>1</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>12018</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -976,11 +1208,15 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" t="n">
-        <v>12019</v>
-      </c>
-      <c r="C20" t="n">
-        <v>1</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>12019</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1004,11 +1240,15 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" t="n">
-        <v>12021</v>
-      </c>
-      <c r="C21" t="n">
-        <v>1</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>12021</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1032,11 +1272,15 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" t="n">
-        <v>12023</v>
-      </c>
-      <c r="C22" t="n">
-        <v>1</v>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>12023</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1060,11 +1304,15 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" t="n">
-        <v>12024</v>
-      </c>
-      <c r="C23" t="n">
-        <v>1</v>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>12024</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1088,11 +1336,15 @@
       </c>
     </row>
     <row r="24">
-      <c r="B24" t="n">
-        <v>12025</v>
-      </c>
-      <c r="C24" t="n">
-        <v>1</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>12025</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1116,11 +1368,15 @@
       </c>
     </row>
     <row r="25">
-      <c r="B25" t="n">
-        <v>12027</v>
-      </c>
-      <c r="C25" t="n">
-        <v>1</v>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>12027</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1144,11 +1400,15 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" t="n">
-        <v>12029</v>
-      </c>
-      <c r="C26" t="n">
-        <v>1</v>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>12029</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1172,11 +1432,15 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" t="n">
-        <v>12030</v>
-      </c>
-      <c r="C27" t="n">
-        <v>1</v>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>12030</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1200,11 +1464,15 @@
       </c>
     </row>
     <row r="28">
-      <c r="B28" t="n">
-        <v>12031</v>
-      </c>
-      <c r="C28" t="n">
-        <v>1</v>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>12031</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1228,11 +1496,15 @@
       </c>
     </row>
     <row r="29">
-      <c r="B29" t="n">
-        <v>12032</v>
-      </c>
-      <c r="C29" t="n">
-        <v>1</v>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>12032</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1256,11 +1528,15 @@
       </c>
     </row>
     <row r="30">
-      <c r="B30" t="n">
-        <v>12036</v>
-      </c>
-      <c r="C30" t="n">
-        <v>1</v>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>12036</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1284,11 +1560,15 @@
       </c>
     </row>
     <row r="31">
-      <c r="B31" t="n">
-        <v>12037</v>
-      </c>
-      <c r="C31" t="n">
-        <v>1</v>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>12037</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1312,11 +1592,15 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" t="n">
-        <v>12038</v>
-      </c>
-      <c r="C32" t="n">
-        <v>1</v>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>12038</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1340,11 +1624,15 @@
       </c>
     </row>
     <row r="33">
-      <c r="B33" t="n">
-        <v>12040</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12040</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1368,11 +1656,15 @@
       </c>
     </row>
     <row r="34">
-      <c r="B34" t="n">
-        <v>12041</v>
-      </c>
-      <c r="C34" t="n">
-        <v>1</v>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>12041</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1396,11 +1688,15 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" t="n">
-        <v>12042</v>
-      </c>
-      <c r="C35" t="n">
-        <v>1</v>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>12042</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1424,11 +1720,15 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" t="n">
-        <v>12044</v>
-      </c>
-      <c r="C36" t="n">
-        <v>1</v>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>12044</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1452,11 +1752,15 @@
       </c>
     </row>
     <row r="37">
-      <c r="B37" t="n">
-        <v>12045</v>
-      </c>
-      <c r="C37" t="n">
-        <v>1</v>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>12045</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1480,11 +1784,15 @@
       </c>
     </row>
     <row r="38">
-      <c r="B38" t="n">
-        <v>12047</v>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>12047</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1508,11 +1816,15 @@
       </c>
     </row>
     <row r="39">
-      <c r="B39" t="n">
-        <v>12048</v>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>12048</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1536,11 +1848,15 @@
       </c>
     </row>
     <row r="40">
-      <c r="B40" t="n">
-        <v>12049</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>12049</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1564,11 +1880,15 @@
       </c>
     </row>
     <row r="41">
-      <c r="B41" t="n">
-        <v>12052</v>
-      </c>
-      <c r="C41" t="n">
-        <v>1</v>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>12052</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1592,11 +1912,15 @@
       </c>
     </row>
     <row r="42">
-      <c r="B42" t="n">
-        <v>12053</v>
-      </c>
-      <c r="C42" t="n">
-        <v>1</v>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>12053</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1620,11 +1944,15 @@
       </c>
     </row>
     <row r="43">
-      <c r="B43" t="n">
-        <v>12055</v>
-      </c>
-      <c r="C43" t="n">
-        <v>1</v>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>12055</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1648,11 +1976,15 @@
       </c>
     </row>
     <row r="44">
-      <c r="B44" t="n">
-        <v>12057</v>
-      </c>
-      <c r="C44" t="n">
-        <v>1</v>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>12057</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1676,11 +2008,15 @@
       </c>
     </row>
     <row r="45">
-      <c r="B45" t="n">
-        <v>12058</v>
-      </c>
-      <c r="C45" t="n">
-        <v>1</v>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>12058</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1704,11 +2040,15 @@
       </c>
     </row>
     <row r="46">
-      <c r="B46" t="n">
-        <v>12059</v>
-      </c>
-      <c r="C46" t="n">
-        <v>1</v>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>12059</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1732,11 +2072,15 @@
       </c>
     </row>
     <row r="47">
-      <c r="B47" t="n">
-        <v>12060</v>
-      </c>
-      <c r="C47" t="n">
-        <v>1</v>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>12060</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1760,11 +2104,15 @@
       </c>
     </row>
     <row r="48">
-      <c r="B48" t="n">
-        <v>12062</v>
-      </c>
-      <c r="C48" t="n">
-        <v>1</v>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>12062</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1788,11 +2136,15 @@
       </c>
     </row>
     <row r="49">
-      <c r="B49" t="n">
-        <v>12063</v>
-      </c>
-      <c r="C49" t="n">
-        <v>1</v>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>12063</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1982,6 +2334,16 @@
           <t>PerTarget</t>
         </is>
       </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="B56" t="n">
@@ -2010,6 +2372,16 @@
           <t>PerTarget</t>
         </is>
       </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="B57" t="n">
@@ -2038,6 +2410,16 @@
           <t>PerTarget</t>
         </is>
       </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="B58" t="n">
@@ -2066,6 +2448,16 @@
           <t>PerTarget</t>
         </is>
       </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="B59" t="n">
@@ -2094,6 +2486,16 @@
           <t>PerTarget</t>
         </is>
       </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="B60" t="n">
@@ -2542,6 +2944,21 @@
           <t>PerTarget</t>
         </is>
       </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="B76" t="n">
@@ -2570,6 +2987,21 @@
           <t>PerTarget</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>parameter.03</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="B77" t="n">
@@ -3020,6 +3452,18 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="C8:C1007" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 100." promptTitle="Integer range" prompt="Enter an integer from 1 to 100." type="whole">
+      <formula1>1</formula1>
+      <formula2>100</formula2>
+    </dataValidation>
+    <dataValidation sqref="D8:D1007" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid enum value" error="Value must be one of: Primary, Adjacent, Selected, All, BounceDraw, SelfTarget" promptTitle="HitTargetGroup enum" prompt="Select a value from the dropdown." type="list">
+      <formula1>"Primary,Adjacent,Selected,All,BounceDraw,SelfTarget"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G8:G1007" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid enum value" error="Value must be one of: PerTarget, Shared, Never" promptTitle="CritPolicy enum" prompt="Select a value from the dropdown." type="list">
+      <formula1>"PerTarget,Shared,Never"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>